<commit_message>
Fix: Zellformat 0,00 -> 0.00, damit Stunden als 8,40 statt 008 erscheinen
xlsx speichert Zahlenformate in US-Notation. '0,00' bedeutet dort
Tausendertrenner und Excel zeigte jeden Stundenwert gerundet als 008/009/006.
Das Format kam aus der Vorlage und wurde ungeprueft uebernommen.
fix_number_formats() stellt nach dem Schreiben alle '0,00'-Zellen auf '0.00'
um; deutsches Excel zeigt das als 8,40.

Rufat September 2026 neu erzeugt und geprueft: keine 0,00-Zellen mehr,
alle Arbeitszeiten in 5-Minuten-Schritten, Krankheit 18.-25.09.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YVFKXyc2wFgzZv9BeWR84Y
</commit_message>
<xml_diff>
--- a/vma_september_2026_entwurf/Zeiterfassung_September_2026_Rufat_fertig.xlsx
+++ b/vma_september_2026_entwurf/Zeiterfassung_September_2026_Rufat_fertig.xlsx
@@ -247,7 +247,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -409,9 +409,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0"/>
@@ -658,7 +656,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:AG34"/>
+  <dimension ref="A1:AG34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
   <cols>
     <col width="26.875" customWidth="1" style="63" min="1" max="1"/>
@@ -667,6 +665,7 @@
     <col width="8.625" customWidth="1" style="63" min="33" max="33"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="D2" s="79" t="inlineStr">
         <is>
@@ -712,6 +711,8 @@
       <c r="K4" s="75" t="n"/>
       <c r="L4" s="75" t="n"/>
     </row>
+    <row r="5"/>
+    <row r="6"/>
     <row r="7">
       <c r="N7">
         <f>SUM(W7)</f>
@@ -751,6 +752,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11" hidden="1" s="63"/>
     <row r="12" ht="30" customHeight="1" s="63">
       <c r="A12" s="70" t="inlineStr">
@@ -1026,70 +1028,70 @@
           <t>Arbeitszeit</t>
         </is>
       </c>
-      <c r="B14" s="95" t="n">
+      <c r="B14" s="71" t="n">
         <v>8.4</v>
       </c>
-      <c r="C14" s="95" t="n">
+      <c r="C14" s="71" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="D14" s="71" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="E14" s="71" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="F14" s="71" t="n"/>
+      <c r="G14" s="71" t="n"/>
+      <c r="H14" s="71" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="I14" s="71" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="J14" s="71" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="K14" s="71" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="L14" s="71" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="M14" s="71" t="n"/>
+      <c r="N14" s="71" t="n"/>
+      <c r="O14" s="71" t="n">
+        <v>8.449999999999999</v>
+      </c>
+      <c r="P14" s="71" t="n">
+        <v>8.35</v>
+      </c>
+      <c r="Q14" s="71" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="R14" s="71" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="S14" s="71" t="n"/>
+      <c r="T14" s="71" t="n"/>
+      <c r="U14" s="71" t="n"/>
+      <c r="V14" s="71" t="n"/>
+      <c r="W14" s="71" t="n"/>
+      <c r="X14" s="71" t="n"/>
+      <c r="Y14" s="71" t="n"/>
+      <c r="Z14" s="71" t="n"/>
+      <c r="AA14" s="71" t="n"/>
+      <c r="AB14" s="71" t="n"/>
+      <c r="AC14" s="71" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="AD14" s="71" t="n">
+        <v>8.199999999999999</v>
+      </c>
+      <c r="AE14" s="71" t="n">
         <v>8.4</v>
       </c>
-      <c r="D14" s="95" t="n">
-        <v>8.449999999999999</v>
-      </c>
-      <c r="E14" s="95" t="n">
-        <v>8.4</v>
-      </c>
-      <c r="F14" s="95" t="n"/>
-      <c r="G14" s="95" t="n"/>
-      <c r="H14" s="95" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="I14" s="95" t="n">
-        <v>8.15</v>
-      </c>
-      <c r="J14" s="95" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="K14" s="95" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="L14" s="95" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="M14" s="95" t="n"/>
-      <c r="N14" s="95" t="n"/>
-      <c r="O14" s="95" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="P14" s="95" t="n">
-        <v>9</v>
-      </c>
-      <c r="Q14" s="95" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="R14" s="95" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="S14" s="95" t="n"/>
-      <c r="T14" s="95" t="n"/>
-      <c r="U14" s="95" t="n"/>
-      <c r="V14" s="95" t="n"/>
-      <c r="W14" s="95" t="n"/>
-      <c r="X14" s="95" t="n"/>
-      <c r="Y14" s="95" t="n"/>
-      <c r="Z14" s="95" t="n"/>
-      <c r="AA14" s="95" t="n"/>
-      <c r="AB14" s="95" t="n"/>
-      <c r="AC14" s="95" t="n">
-        <v>8.449999999999999</v>
-      </c>
-      <c r="AD14" s="95" t="n">
-        <v>8.35</v>
-      </c>
-      <c r="AE14" s="95" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="AF14" s="95" t="n"/>
-      <c r="AG14" s="95">
+      <c r="AF14" s="71" t="n"/>
+      <c r="AG14" s="71">
         <f>SUM(B14:AF14)</f>
         <v/>
       </c>
@@ -1100,38 +1102,38 @@
           <t>bez. Urlaub</t>
         </is>
       </c>
-      <c r="B15" s="95" t="n"/>
-      <c r="C15" s="95" t="n"/>
-      <c r="D15" s="95" t="n"/>
-      <c r="E15" s="95" t="n"/>
-      <c r="F15" s="95" t="n"/>
-      <c r="G15" s="95" t="n"/>
-      <c r="H15" s="95" t="n"/>
-      <c r="I15" s="95" t="n"/>
-      <c r="J15" s="95" t="n"/>
-      <c r="K15" s="95" t="n"/>
-      <c r="L15" s="95" t="n"/>
-      <c r="M15" s="95" t="n"/>
-      <c r="N15" s="95" t="n"/>
-      <c r="O15" s="95" t="n"/>
-      <c r="P15" s="95" t="n"/>
-      <c r="Q15" s="95" t="n"/>
-      <c r="R15" s="95" t="n"/>
-      <c r="S15" s="95" t="n"/>
-      <c r="T15" s="95" t="n"/>
-      <c r="U15" s="95" t="n"/>
-      <c r="V15" s="95" t="n"/>
-      <c r="W15" s="95" t="n"/>
-      <c r="X15" s="95" t="n"/>
-      <c r="Y15" s="95" t="n"/>
-      <c r="Z15" s="95" t="n"/>
-      <c r="AA15" s="95" t="n"/>
-      <c r="AB15" s="95" t="n"/>
-      <c r="AC15" s="95" t="n"/>
-      <c r="AD15" s="95" t="n"/>
-      <c r="AE15" s="95" t="n"/>
-      <c r="AF15" s="95" t="n"/>
-      <c r="AG15" s="95">
+      <c r="B15" s="71" t="n"/>
+      <c r="C15" s="71" t="n"/>
+      <c r="D15" s="71" t="n"/>
+      <c r="E15" s="71" t="n"/>
+      <c r="F15" s="71" t="n"/>
+      <c r="G15" s="71" t="n"/>
+      <c r="H15" s="71" t="n"/>
+      <c r="I15" s="71" t="n"/>
+      <c r="J15" s="71" t="n"/>
+      <c r="K15" s="71" t="n"/>
+      <c r="L15" s="71" t="n"/>
+      <c r="M15" s="71" t="n"/>
+      <c r="N15" s="71" t="n"/>
+      <c r="O15" s="71" t="n"/>
+      <c r="P15" s="71" t="n"/>
+      <c r="Q15" s="71" t="n"/>
+      <c r="R15" s="71" t="n"/>
+      <c r="S15" s="71" t="n"/>
+      <c r="T15" s="71" t="n"/>
+      <c r="U15" s="71" t="n"/>
+      <c r="V15" s="71" t="n"/>
+      <c r="W15" s="71" t="n"/>
+      <c r="X15" s="71" t="n"/>
+      <c r="Y15" s="71" t="n"/>
+      <c r="Z15" s="71" t="n"/>
+      <c r="AA15" s="71" t="n"/>
+      <c r="AB15" s="71" t="n"/>
+      <c r="AC15" s="71" t="n"/>
+      <c r="AD15" s="71" t="n"/>
+      <c r="AE15" s="71" t="n"/>
+      <c r="AF15" s="71" t="n"/>
+      <c r="AG15" s="71">
         <f>SUM(B15:AF15)</f>
         <v/>
       </c>
@@ -1142,131 +1144,131 @@
           <t>Feiertage</t>
         </is>
       </c>
-      <c r="B16" s="95">
+      <c r="B16" s="71">
         <f>IF(B$12="","","-")</f>
         <v/>
       </c>
-      <c r="C16" s="95">
+      <c r="C16" s="71">
         <f>IF(C$12="","","-")</f>
         <v/>
       </c>
-      <c r="D16" s="95">
+      <c r="D16" s="71">
         <f>IF(D$12="","","-")</f>
         <v/>
       </c>
-      <c r="E16" s="95">
+      <c r="E16" s="71">
         <f>IF(E$12="","","-")</f>
         <v/>
       </c>
-      <c r="F16" s="95">
+      <c r="F16" s="71">
         <f>IF(F$12="","","-")</f>
         <v/>
       </c>
-      <c r="G16" s="95">
+      <c r="G16" s="71">
         <f>IF(G$12="","","-")</f>
         <v/>
       </c>
-      <c r="H16" s="95">
+      <c r="H16" s="71">
         <f>IF(H$12="","","-")</f>
         <v/>
       </c>
-      <c r="I16" s="95">
+      <c r="I16" s="71">
         <f>IF(I$12="","","-")</f>
         <v/>
       </c>
-      <c r="J16" s="95">
+      <c r="J16" s="71">
         <f>IF(J$12="","","-")</f>
         <v/>
       </c>
-      <c r="K16" s="95">
+      <c r="K16" s="71">
         <f>IF(K$12="","","-")</f>
         <v/>
       </c>
-      <c r="L16" s="95">
+      <c r="L16" s="71">
         <f>IF(L$12="","","-")</f>
         <v/>
       </c>
-      <c r="M16" s="95">
+      <c r="M16" s="71">
         <f>IF(M$12="","","-")</f>
         <v/>
       </c>
-      <c r="N16" s="95">
+      <c r="N16" s="71">
         <f>IF(N$12="","","-")</f>
         <v/>
       </c>
-      <c r="O16" s="95">
+      <c r="O16" s="71">
         <f>IF(O$12="","","-")</f>
         <v/>
       </c>
-      <c r="P16" s="95">
+      <c r="P16" s="71">
         <f>IF(P$12="","","-")</f>
         <v/>
       </c>
-      <c r="Q16" s="95">
+      <c r="Q16" s="71">
         <f>IF(Q$12="","","-")</f>
         <v/>
       </c>
-      <c r="R16" s="95">
+      <c r="R16" s="71">
         <f>IF(R$12="","","-")</f>
         <v/>
       </c>
-      <c r="S16" s="95">
+      <c r="S16" s="71">
         <f>IF(S$12="","","-")</f>
         <v/>
       </c>
-      <c r="T16" s="95">
+      <c r="T16" s="71">
         <f>IF(T$12="","","-")</f>
         <v/>
       </c>
-      <c r="U16" s="95">
+      <c r="U16" s="71">
         <f>IF(U$12="","","-")</f>
         <v/>
       </c>
-      <c r="V16" s="95">
+      <c r="V16" s="71">
         <f>IF(V$12="","","-")</f>
         <v/>
       </c>
-      <c r="W16" s="95">
+      <c r="W16" s="71">
         <f>IF(W$12="","","-")</f>
         <v/>
       </c>
-      <c r="X16" s="95">
+      <c r="X16" s="71">
         <f>IF(X$12="","","-")</f>
         <v/>
       </c>
-      <c r="Y16" s="95">
+      <c r="Y16" s="71">
         <f>IF(Y$12="","","-")</f>
         <v/>
       </c>
-      <c r="Z16" s="95">
+      <c r="Z16" s="71">
         <f>IF(Z$12="","","-")</f>
         <v/>
       </c>
-      <c r="AA16" s="95">
+      <c r="AA16" s="71">
         <f>IF(AA$12="","","-")</f>
         <v/>
       </c>
-      <c r="AB16" s="95">
+      <c r="AB16" s="71">
         <f>IF(AB$12="","","-")</f>
         <v/>
       </c>
-      <c r="AC16" s="95">
+      <c r="AC16" s="71">
         <f>IF(AC$12="","","-")</f>
         <v/>
       </c>
-      <c r="AD16" s="95">
+      <c r="AD16" s="71">
         <f>IF(AD$12="","","-")</f>
         <v/>
       </c>
-      <c r="AE16" s="95">
+      <c r="AE16" s="71">
         <f>IF(AE$12="","","-")</f>
         <v/>
       </c>
-      <c r="AF16" s="95">
+      <c r="AF16" s="71">
         <f>IF(AF$12="","","-")</f>
         <v/>
       </c>
-      <c r="AG16" s="95">
+      <c r="AG16" s="71">
         <f>SUM(B16:AF16)</f>
         <v/>
       </c>
@@ -1277,123 +1279,123 @@
           <t>Krankentage</t>
         </is>
       </c>
-      <c r="B17" s="95">
+      <c r="B17" s="71">
         <f>IF(B$12="","","-")</f>
         <v/>
       </c>
-      <c r="C17" s="95">
+      <c r="C17" s="71">
         <f>IF(C$12="","","-")</f>
         <v/>
       </c>
-      <c r="D17" s="95">
+      <c r="D17" s="71">
         <f>IF(D$12="","","-")</f>
         <v/>
       </c>
-      <c r="E17" s="95">
+      <c r="E17" s="71">
         <f>IF(E$12="","","-")</f>
         <v/>
       </c>
-      <c r="F17" s="95">
+      <c r="F17" s="71">
         <f>IF(F$12="","","-")</f>
         <v/>
       </c>
-      <c r="G17" s="95">
+      <c r="G17" s="71">
         <f>IF(G$12="","","-")</f>
         <v/>
       </c>
-      <c r="H17" s="95">
+      <c r="H17" s="71">
         <f>IF(H$12="","","-")</f>
         <v/>
       </c>
-      <c r="I17" s="95">
+      <c r="I17" s="71">
         <f>IF(I$12="","","-")</f>
         <v/>
       </c>
-      <c r="J17" s="95">
+      <c r="J17" s="71">
         <f>IF(J$12="","","-")</f>
         <v/>
       </c>
-      <c r="K17" s="95">
+      <c r="K17" s="71">
         <f>IF(K$12="","","-")</f>
         <v/>
       </c>
-      <c r="L17" s="95">
+      <c r="L17" s="71">
         <f>IF(L$12="","","-")</f>
         <v/>
       </c>
-      <c r="M17" s="95">
+      <c r="M17" s="71">
         <f>IF(M$12="","","-")</f>
         <v/>
       </c>
-      <c r="N17" s="95">
+      <c r="N17" s="71">
         <f>IF(N$12="","","-")</f>
         <v/>
       </c>
-      <c r="O17" s="95">
+      <c r="O17" s="71">
         <f>IF(O$12="","","-")</f>
         <v/>
       </c>
-      <c r="P17" s="95">
+      <c r="P17" s="71">
         <f>IF(P$12="","","-")</f>
         <v/>
       </c>
-      <c r="Q17" s="95">
+      <c r="Q17" s="71">
         <f>IF(Q$12="","","-")</f>
         <v/>
       </c>
-      <c r="R17" s="95">
+      <c r="R17" s="71">
         <f>IF(R$12="","","-")</f>
         <v/>
       </c>
-      <c r="S17" s="95" t="n">
+      <c r="S17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="T17" s="95" t="n">
+      <c r="T17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="U17" s="95" t="n">
+      <c r="U17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="V17" s="95" t="n">
+      <c r="V17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="W17" s="95" t="n">
+      <c r="W17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="X17" s="95" t="n">
+      <c r="X17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="Y17" s="95" t="n">
+      <c r="Y17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="Z17" s="95" t="n">
+      <c r="Z17" s="71" t="n">
         <v>8</v>
       </c>
-      <c r="AA17" s="95">
+      <c r="AA17" s="71">
         <f>IF(AA$12="","","-")</f>
         <v/>
       </c>
-      <c r="AB17" s="95">
+      <c r="AB17" s="71">
         <f>IF(AB$12="","","-")</f>
         <v/>
       </c>
-      <c r="AC17" s="95">
+      <c r="AC17" s="71">
         <f>IF(AC$12="","","-")</f>
         <v/>
       </c>
-      <c r="AD17" s="95">
+      <c r="AD17" s="71">
         <f>IF(AD$12="","","-")</f>
         <v/>
       </c>
-      <c r="AE17" s="95">
+      <c r="AE17" s="71">
         <f>IF(AE$12="","","-")</f>
         <v/>
       </c>
-      <c r="AF17" s="95">
+      <c r="AF17" s="71">
         <f>IF(AF$12="","","-")</f>
         <v/>
       </c>
-      <c r="AG17" s="95">
+      <c r="AG17" s="71">
         <f>SUM(B17:AF17)</f>
         <v/>
       </c>
@@ -1404,131 +1406,131 @@
           <t>Sonstige Fehlzeiten</t>
         </is>
       </c>
-      <c r="B18" s="95">
+      <c r="B18" s="71">
         <f>IF(B$12="","","-")</f>
         <v/>
       </c>
-      <c r="C18" s="95">
+      <c r="C18" s="71">
         <f>IF(C$12="","","-")</f>
         <v/>
       </c>
-      <c r="D18" s="95">
+      <c r="D18" s="71">
         <f>IF(D$12="","","-")</f>
         <v/>
       </c>
-      <c r="E18" s="95">
+      <c r="E18" s="71">
         <f>IF(E$12="","","-")</f>
         <v/>
       </c>
-      <c r="F18" s="95">
+      <c r="F18" s="71">
         <f>IF(F$12="","","-")</f>
         <v/>
       </c>
-      <c r="G18" s="95">
+      <c r="G18" s="71">
         <f>IF(G$12="","","-")</f>
         <v/>
       </c>
-      <c r="H18" s="95">
+      <c r="H18" s="71">
         <f>IF(H$12="","","-")</f>
         <v/>
       </c>
-      <c r="I18" s="95">
+      <c r="I18" s="71">
         <f>IF(I$12="","","-")</f>
         <v/>
       </c>
-      <c r="J18" s="95">
+      <c r="J18" s="71">
         <f>IF(J$12="","","-")</f>
         <v/>
       </c>
-      <c r="K18" s="95">
+      <c r="K18" s="71">
         <f>IF(K$12="","","-")</f>
         <v/>
       </c>
-      <c r="L18" s="95">
+      <c r="L18" s="71">
         <f>IF(L$12="","","-")</f>
         <v/>
       </c>
-      <c r="M18" s="95">
+      <c r="M18" s="71">
         <f>IF(M$12="","","-")</f>
         <v/>
       </c>
-      <c r="N18" s="95">
+      <c r="N18" s="71">
         <f>IF(N$12="","","-")</f>
         <v/>
       </c>
-      <c r="O18" s="95">
+      <c r="O18" s="71">
         <f>IF(O$12="","","-")</f>
         <v/>
       </c>
-      <c r="P18" s="95">
+      <c r="P18" s="71">
         <f>IF(P$12="","","-")</f>
         <v/>
       </c>
-      <c r="Q18" s="95">
+      <c r="Q18" s="71">
         <f>IF(Q$12="","","-")</f>
         <v/>
       </c>
-      <c r="R18" s="95">
+      <c r="R18" s="71">
         <f>IF(R$12="","","-")</f>
         <v/>
       </c>
-      <c r="S18" s="95">
+      <c r="S18" s="71">
         <f>IF(S$12="","","-")</f>
         <v/>
       </c>
-      <c r="T18" s="95">
+      <c r="T18" s="71">
         <f>IF(T$12="","","-")</f>
         <v/>
       </c>
-      <c r="U18" s="95">
+      <c r="U18" s="71">
         <f>IF(U$12="","","-")</f>
         <v/>
       </c>
-      <c r="V18" s="95">
+      <c r="V18" s="71">
         <f>IF(V$12="","","-")</f>
         <v/>
       </c>
-      <c r="W18" s="95">
+      <c r="W18" s="71">
         <f>IF(W$12="","","-")</f>
         <v/>
       </c>
-      <c r="X18" s="95">
+      <c r="X18" s="71">
         <f>IF(X$12="","","-")</f>
         <v/>
       </c>
-      <c r="Y18" s="95">
+      <c r="Y18" s="71">
         <f>IF(Y$12="","","-")</f>
         <v/>
       </c>
-      <c r="Z18" s="95">
+      <c r="Z18" s="71">
         <f>IF(Z$12="","","-")</f>
         <v/>
       </c>
-      <c r="AA18" s="95">
+      <c r="AA18" s="71">
         <f>IF(AA$12="","","-")</f>
         <v/>
       </c>
-      <c r="AB18" s="95">
+      <c r="AB18" s="71">
         <f>IF(AB$12="","","-")</f>
         <v/>
       </c>
-      <c r="AC18" s="95">
+      <c r="AC18" s="71">
         <f>IF(AC$12="","","-")</f>
         <v/>
       </c>
-      <c r="AD18" s="95">
+      <c r="AD18" s="71">
         <f>IF(AD$12="","","-")</f>
         <v/>
       </c>
-      <c r="AE18" s="95">
+      <c r="AE18" s="71">
         <f>IF(AE$12="","","-")</f>
         <v/>
       </c>
-      <c r="AF18" s="95">
+      <c r="AF18" s="71">
         <f>IF(AF$12="","","-")</f>
         <v/>
       </c>
-      <c r="AG18" s="95">
+      <c r="AG18" s="71">
         <f>SUM(B18:AF18)</f>
         <v/>
       </c>
@@ -1539,38 +1541,38 @@
           <t>Gesamt-Stunden</t>
         </is>
       </c>
-      <c r="B19" s="95" t="n"/>
-      <c r="C19" s="95" t="n"/>
-      <c r="D19" s="95" t="n"/>
-      <c r="E19" s="95" t="n"/>
-      <c r="F19" s="95" t="n"/>
-      <c r="G19" s="95" t="n"/>
-      <c r="H19" s="95" t="n"/>
-      <c r="I19" s="95" t="n"/>
-      <c r="J19" s="95" t="n"/>
-      <c r="K19" s="95" t="n"/>
-      <c r="L19" s="95" t="n"/>
-      <c r="M19" s="95" t="n"/>
-      <c r="N19" s="95" t="n"/>
-      <c r="O19" s="95" t="n"/>
-      <c r="P19" s="95" t="n"/>
-      <c r="Q19" s="95" t="n"/>
-      <c r="R19" s="95" t="n"/>
-      <c r="S19" s="95" t="n"/>
-      <c r="T19" s="95" t="n"/>
-      <c r="U19" s="95" t="n"/>
-      <c r="V19" s="95" t="n"/>
-      <c r="W19" s="95" t="n"/>
-      <c r="X19" s="95" t="n"/>
-      <c r="Y19" s="95" t="n"/>
-      <c r="Z19" s="95" t="n"/>
-      <c r="AA19" s="95" t="n"/>
-      <c r="AB19" s="95" t="n"/>
-      <c r="AC19" s="95" t="n"/>
-      <c r="AD19" s="95" t="n"/>
-      <c r="AE19" s="95" t="n"/>
-      <c r="AF19" s="95" t="n"/>
-      <c r="AG19" s="95">
+      <c r="B19" s="71" t="n"/>
+      <c r="C19" s="71" t="n"/>
+      <c r="D19" s="71" t="n"/>
+      <c r="E19" s="71" t="n"/>
+      <c r="F19" s="71" t="n"/>
+      <c r="G19" s="71" t="n"/>
+      <c r="H19" s="71" t="n"/>
+      <c r="I19" s="71" t="n"/>
+      <c r="J19" s="71" t="n"/>
+      <c r="K19" s="71" t="n"/>
+      <c r="L19" s="71" t="n"/>
+      <c r="M19" s="71" t="n"/>
+      <c r="N19" s="71" t="n"/>
+      <c r="O19" s="71" t="n"/>
+      <c r="P19" s="71" t="n"/>
+      <c r="Q19" s="71" t="n"/>
+      <c r="R19" s="71" t="n"/>
+      <c r="S19" s="71" t="n"/>
+      <c r="T19" s="71" t="n"/>
+      <c r="U19" s="71" t="n"/>
+      <c r="V19" s="71" t="n"/>
+      <c r="W19" s="71" t="n"/>
+      <c r="X19" s="71" t="n"/>
+      <c r="Y19" s="71" t="n"/>
+      <c r="Z19" s="71" t="n"/>
+      <c r="AA19" s="71" t="n"/>
+      <c r="AB19" s="71" t="n"/>
+      <c r="AC19" s="71" t="n"/>
+      <c r="AD19" s="71" t="n"/>
+      <c r="AE19" s="71" t="n"/>
+      <c r="AF19" s="71" t="n"/>
+      <c r="AG19" s="71">
         <f>SUM(AG14:AG18)</f>
         <v/>
       </c>
@@ -1581,131 +1583,131 @@
           <t>VMA-Tag (1=ja)</t>
         </is>
       </c>
-      <c r="B20" s="96">
+      <c r="B20" s="95">
         <f>IF(B12="","",IF(B14="-","-",IF(B14="","",IF(AND(ISNUMBER(B14),INT(B14)*100+ROUND(MOD(B14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="C20" s="96">
+      <c r="C20" s="95">
         <f>IF(C12="","",IF(C14="-","-",IF(C14="","",IF(AND(ISNUMBER(C14),INT(C14)*100+ROUND(MOD(C14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="D20" s="96">
+      <c r="D20" s="95">
         <f>IF(D12="","",IF(D14="-","-",IF(D14="","",IF(AND(ISNUMBER(D14),INT(D14)*100+ROUND(MOD(D14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="E20" s="96">
+      <c r="E20" s="95">
         <f>IF(E12="","",IF(E14="-","-",IF(E14="","",IF(AND(ISNUMBER(E14),INT(E14)*100+ROUND(MOD(E14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="F20" s="96">
+      <c r="F20" s="95">
         <f>IF(F12="","",IF(F14="-","-",IF(F14="","",IF(AND(ISNUMBER(F14),INT(F14)*100+ROUND(MOD(F14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="G20" s="96">
+      <c r="G20" s="95">
         <f>IF(G12="","",IF(G14="-","-",IF(G14="","",IF(AND(ISNUMBER(G14),INT(G14)*100+ROUND(MOD(G14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="H20" s="96">
+      <c r="H20" s="95">
         <f>IF(H12="","",IF(H14="-","-",IF(H14="","",IF(AND(ISNUMBER(H14),INT(H14)*100+ROUND(MOD(H14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="I20" s="96">
+      <c r="I20" s="95">
         <f>IF(I12="","",IF(I14="-","-",IF(I14="","",IF(AND(ISNUMBER(I14),INT(I14)*100+ROUND(MOD(I14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="J20" s="96">
+      <c r="J20" s="95">
         <f>IF(J12="","",IF(J14="-","-",IF(J14="","",IF(AND(ISNUMBER(J14),INT(J14)*100+ROUND(MOD(J14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="K20" s="96">
+      <c r="K20" s="95">
         <f>IF(K12="","",IF(K14="-","-",IF(K14="","",IF(AND(ISNUMBER(K14),INT(K14)*100+ROUND(MOD(K14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="L20" s="96">
+      <c r="L20" s="95">
         <f>IF(L12="","",IF(L14="-","-",IF(L14="","",IF(AND(ISNUMBER(L14),INT(L14)*100+ROUND(MOD(L14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="M20" s="96">
+      <c r="M20" s="95">
         <f>IF(M12="","",IF(M14="-","-",IF(M14="","",IF(AND(ISNUMBER(M14),INT(M14)*100+ROUND(MOD(M14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="N20" s="96">
+      <c r="N20" s="95">
         <f>IF(N12="","",IF(N14="-","-",IF(N14="","",IF(AND(ISNUMBER(N14),INT(N14)*100+ROUND(MOD(N14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="O20" s="96">
+      <c r="O20" s="95">
         <f>IF(O12="","",IF(O14="-","-",IF(O14="","",IF(AND(ISNUMBER(O14),INT(O14)*100+ROUND(MOD(O14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="P20" s="96">
+      <c r="P20" s="95">
         <f>IF(P12="","",IF(P14="-","-",IF(P14="","",IF(AND(ISNUMBER(P14),INT(P14)*100+ROUND(MOD(P14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="Q20" s="96">
+      <c r="Q20" s="95">
         <f>IF(Q12="","",IF(Q14="-","-",IF(Q14="","",IF(AND(ISNUMBER(Q14),INT(Q14)*100+ROUND(MOD(Q14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="R20" s="96">
+      <c r="R20" s="95">
         <f>IF(R12="","",IF(R14="-","-",IF(R14="","",IF(AND(ISNUMBER(R14),INT(R14)*100+ROUND(MOD(R14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="S20" s="96">
+      <c r="S20" s="95">
         <f>IF(S12="","",IF(S14="-","-",IF(S14="","",IF(AND(ISNUMBER(S14),INT(S14)*100+ROUND(MOD(S14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="T20" s="96">
+      <c r="T20" s="95">
         <f>IF(T12="","",IF(T14="-","-",IF(T14="","",IF(AND(ISNUMBER(T14),INT(T14)*100+ROUND(MOD(T14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="U20" s="96">
+      <c r="U20" s="95">
         <f>IF(U12="","",IF(U14="-","-",IF(U14="","",IF(AND(ISNUMBER(U14),INT(U14)*100+ROUND(MOD(U14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="V20" s="96">
+      <c r="V20" s="95">
         <f>IF(V12="","",IF(V14="-","-",IF(V14="","",IF(AND(ISNUMBER(V14),INT(V14)*100+ROUND(MOD(V14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="W20" s="96">
+      <c r="W20" s="95">
         <f>IF(W12="","",IF(W14="-","-",IF(W14="","",IF(AND(ISNUMBER(W14),INT(W14)*100+ROUND(MOD(W14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="X20" s="96">
+      <c r="X20" s="95">
         <f>IF(X12="","",IF(X14="-","-",IF(X14="","",IF(AND(ISNUMBER(X14),INT(X14)*100+ROUND(MOD(X14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="Y20" s="96">
+      <c r="Y20" s="95">
         <f>IF(Y12="","",IF(Y14="-","-",IF(Y14="","",IF(AND(ISNUMBER(Y14),INT(Y14)*100+ROUND(MOD(Y14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="Z20" s="96">
+      <c r="Z20" s="95">
         <f>IF(Z12="","",IF(Z14="-","-",IF(Z14="","",IF(AND(ISNUMBER(Z14),INT(Z14)*100+ROUND(MOD(Z14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AA20" s="96">
+      <c r="AA20" s="95">
         <f>IF(AA12="","",IF(AA14="-","-",IF(AA14="","",IF(AND(ISNUMBER(AA14),INT(AA14)*100+ROUND(MOD(AA14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AB20" s="96">
+      <c r="AB20" s="95">
         <f>IF(AB12="","",IF(AB14="-","-",IF(AB14="","",IF(AND(ISNUMBER(AB14),INT(AB14)*100+ROUND(MOD(AB14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AC20" s="96">
+      <c r="AC20" s="95">
         <f>IF(AC12="","",IF(AC14="-","-",IF(AC14="","",IF(AND(ISNUMBER(AC14),INT(AC14)*100+ROUND(MOD(AC14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AD20" s="96">
+      <c r="AD20" s="95">
         <f>IF(AD12="","",IF(AD14="-","-",IF(AD14="","",IF(AND(ISNUMBER(AD14),INT(AD14)*100+ROUND(MOD(AD14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AE20" s="96">
+      <c r="AE20" s="95">
         <f>IF(AE12="","",IF(AE14="-","-",IF(AE14="","",IF(AND(ISNUMBER(AE14),INT(AE14)*100+ROUND(MOD(AE14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AF20" s="96">
+      <c r="AF20" s="95">
         <f>IF(AF12="","",IF(AF14="-","-",IF(AF14="","",IF(AND(ISNUMBER(AF14),INT(AF14)*100+ROUND(MOD(AF14,1)*100,0)&gt;800),1,"-"))))</f>
         <v/>
       </c>
-      <c r="AG20" s="96">
+      <c r="AG20" s="95">
         <f>SUM(B20:AF20)</f>
         <v/>
       </c>
@@ -1716,135 +1718,136 @@
           <t>VMA €</t>
         </is>
       </c>
-      <c r="B21" s="95">
+      <c r="B21" s="71">
         <f>IF(B20=1,14,0)</f>
         <v/>
       </c>
-      <c r="C21" s="95">
+      <c r="C21" s="71">
         <f>IF(C20=1,14,0)</f>
         <v/>
       </c>
-      <c r="D21" s="95">
+      <c r="D21" s="71">
         <f>IF(D20=1,14,0)</f>
         <v/>
       </c>
-      <c r="E21" s="95">
+      <c r="E21" s="71">
         <f>IF(E20=1,14,0)</f>
         <v/>
       </c>
-      <c r="F21" s="95">
+      <c r="F21" s="71">
         <f>IF(F20=1,14,0)</f>
         <v/>
       </c>
-      <c r="G21" s="95">
+      <c r="G21" s="71">
         <f>IF(G20=1,14,0)</f>
         <v/>
       </c>
-      <c r="H21" s="95">
+      <c r="H21" s="71">
         <f>IF(H20=1,14,0)</f>
         <v/>
       </c>
-      <c r="I21" s="95">
+      <c r="I21" s="71">
         <f>IF(I20=1,14,0)</f>
         <v/>
       </c>
-      <c r="J21" s="95">
+      <c r="J21" s="71">
         <f>IF(J20=1,14,0)</f>
         <v/>
       </c>
-      <c r="K21" s="95">
+      <c r="K21" s="71">
         <f>IF(K20=1,14,0)</f>
         <v/>
       </c>
-      <c r="L21" s="95">
+      <c r="L21" s="71">
         <f>IF(L20=1,14,0)</f>
         <v/>
       </c>
-      <c r="M21" s="95">
+      <c r="M21" s="71">
         <f>IF(M20=1,14,0)</f>
         <v/>
       </c>
-      <c r="N21" s="95">
+      <c r="N21" s="71">
         <f>IF(N20=1,14,0)</f>
         <v/>
       </c>
-      <c r="O21" s="95">
+      <c r="O21" s="71">
         <f>IF(O20=1,14,0)</f>
         <v/>
       </c>
-      <c r="P21" s="95">
+      <c r="P21" s="71">
         <f>IF(P20=1,14,0)</f>
         <v/>
       </c>
-      <c r="Q21" s="95">
+      <c r="Q21" s="71">
         <f>IF(Q20=1,14,0)</f>
         <v/>
       </c>
-      <c r="R21" s="95">
+      <c r="R21" s="71">
         <f>IF(R20=1,14,0)</f>
         <v/>
       </c>
-      <c r="S21" s="95">
+      <c r="S21" s="71">
         <f>IF(S20=1,14,0)</f>
         <v/>
       </c>
-      <c r="T21" s="95">
+      <c r="T21" s="71">
         <f>IF(T20=1,14,0)</f>
         <v/>
       </c>
-      <c r="U21" s="95">
+      <c r="U21" s="71">
         <f>IF(U20=1,14,0)</f>
         <v/>
       </c>
-      <c r="V21" s="95">
+      <c r="V21" s="71">
         <f>IF(V20=1,14,0)</f>
         <v/>
       </c>
-      <c r="W21" s="95">
+      <c r="W21" s="71">
         <f>IF(W20=1,14,0)</f>
         <v/>
       </c>
-      <c r="X21" s="95">
+      <c r="X21" s="71">
         <f>IF(X20=1,14,0)</f>
         <v/>
       </c>
-      <c r="Y21" s="95">
+      <c r="Y21" s="71">
         <f>IF(Y20=1,14,0)</f>
         <v/>
       </c>
-      <c r="Z21" s="95">
+      <c r="Z21" s="71">
         <f>IF(Z20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AA21" s="95">
+      <c r="AA21" s="71">
         <f>IF(AA20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AB21" s="95">
+      <c r="AB21" s="71">
         <f>IF(AB20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AC21" s="95">
+      <c r="AC21" s="71">
         <f>IF(AC20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AD21" s="95">
+      <c r="AD21" s="71">
         <f>IF(AD20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AE21" s="95">
+      <c r="AE21" s="71">
         <f>IF(AE20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AF21" s="95">
+      <c r="AF21" s="71">
         <f>IF(AF20=1,14,0)</f>
         <v/>
       </c>
-      <c r="AG21" s="95">
+      <c r="AG21" s="71">
         <f>SUM(B21:AF21)</f>
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23" ht="18.75" customHeight="1" s="63">
       <c r="S23" s="53" t="inlineStr">
         <is>
@@ -1872,7 +1875,7 @@
           <t>VMA Satz (€)</t>
         </is>
       </c>
-      <c r="B24" s="95" t="n">
+      <c r="B24" s="71" t="n">
         <v>14</v>
       </c>
       <c r="C24" s="78" t="n"/>
@@ -1913,7 +1916,7 @@
           <t>VMA-Tage (Monat)</t>
         </is>
       </c>
-      <c r="B25" s="97">
+      <c r="B25" s="73">
         <f>AG20</f>
         <v/>
       </c>
@@ -1955,7 +1958,7 @@
           <t>VMA Gesamt (€)</t>
         </is>
       </c>
-      <c r="B26" s="97">
+      <c r="B26" s="73">
         <f>AG21</f>
         <v/>
       </c>

</xml_diff>